<commit_message>
Updated main script and multivariate Bayesian model script to use observed ages only. Sources in Habitat input table updated. Sex ratio map plot revised.
</commit_message>
<xml_diff>
--- a/Input/Habitat.xlsx
+++ b/Input/Habitat.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9888f56ba21a5c62/PostDoc/Analysis/Life-history traits/MedEel LHTs/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9888f56ba21a5c62/PostDoc/Analysis/Life-history traits/Final analysis/MedEel-LHTs/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{F6CB86CA-AFD8-4CBE-B4DE-26FEEB2D7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92E4BC99-5A99-4197-AC66-E3308EDD0DD6}"/>
+  <xr:revisionPtr revIDLastSave="143" documentId="13_ncr:1_{F6CB86CA-AFD8-4CBE-B4DE-26FEEB2D7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A379B89-0E74-4709-A8C0-99D5C72A6444}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" tabRatio="552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Habitat_variables" sheetId="2" r:id="rId1"/>
     <sheet name="Sources" sheetId="4" r:id="rId2"/>
+    <sheet name="README" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Habitat_variables!$A$2:$BW$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sources!$A$2:$D$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sources!$A$2:$D$135</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -986,7 +987,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1773" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="350">
   <si>
     <t>Country</t>
   </si>
@@ -1495,18 +1496,12 @@
     <t>Arnel</t>
   </si>
   <si>
-    <t>FILMED, Gipreb, https://doi.org/10.34930/20384474-8051-4ada-a33d-d16aea5d3a36</t>
-  </si>
-  <si>
     <t>Office de l’Environnement de la Corse</t>
   </si>
   <si>
     <t>Blau, L., &amp; Elger, A. (2020). Suivi de la dynamique des herbiers de zostères dans l’étang du Vaccarès et de la contamination chimique dans les canaux du Fumemorte, du Versadou et du Rousty : Analyse des données pour l’année 2020. Laboratoire Ecologie Fonctionnelle et Environnement, Toulouse. https://www.snpn.com/wp-content/uploads/2021/12/ELGER-2020_Rapport-final_contamination_zost%C3%A8res-Vaccar%C3%A8s.pdf</t>
   </si>
   <si>
-    <t>FILMED network : ADENA, Communauté de communes La Domitienne, EPTB Lez, Gipreb, Maison de la Nature – Ville de Lattes, Perpignan Agglomération, PNR de Camargue, PNR de la Narbonnaise en Méditerranée, SMCG-Syndicat mixte de gestion de la camargue gardoise, SYMBO-Syndicat mixte du bassin de l'or, Syndicat mixte RIVAGE</t>
-  </si>
-  <si>
     <t>Vaccares</t>
   </si>
   <si>
@@ -1615,15 +1610,9 @@
     <t>Sextant and Surval IFREMER database</t>
   </si>
   <si>
-    <t xml:space="preserve">FILMED network : ADENA, Communauté de communes La Domitienne, EPTB Lez, Gipreb, Maison de la Nature – Ville de Lattes, Perpignan Agglomération, PNR de Camargue, PNR de la Narbonnaise en Méditerranée, SMCG-Syndicat mixte de gestion de la camargue gardoise, SYMBO-Syndicat mixte du bassin de l'or, Syndicat mixte RIVAGE; </t>
-  </si>
-  <si>
     <t>Espinosa, C., Abril, M., Bretxa, È., Jutglar, M., Ponsá, S., Sellarès, N., ... &amp; Proia, L. (2021). Driving Factors of Geosmin Appearance in a Mediterranean River Basin: The Ter River Case. Frontiers in Microbiology, 12, 741750. Table 1</t>
   </si>
   <si>
-    <t>Ciccotti, E., Amilhat, E., Bdioui, M., Bendjedid, L., Capoccioni, F., Chebel, F., ... &amp; EB, M. (2023). Towards a range-wide assessment of European eel: recent steps undertaken at the regional scale in the Mediterranean within the GFCM European eel Research Programme, in view of a multiannual Regional management plan.</t>
-  </si>
-  <si>
     <t>Eel GFCM Project</t>
   </si>
   <si>
@@ -1742,9 +1731,6 @@
   </si>
   <si>
     <t>1,72</t>
-  </si>
-  <si>
-    <t>1,70,71,76</t>
   </si>
   <si>
     <t>1,74,75</t>
@@ -3202,7 +3188,296 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Salem, F. B., Said, O. B., Aissa, P., Mahmoudi, E., Monperrus, M., Grunberger, O., &amp; Duran, R. (2016). Pesticides in Ichkeul Lake–Bizerta Lagoon Watershed in Tunisia: use, occurrence, and effects on bacteria and free-living marine nematodes. </t>
+      <t>GÜLÇİÇEK, O. (2018). Investigation of Water Quality of Akgöl Lake in the Göksu Delta. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Advances in Ecological and Environmental Research</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF222222"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 173-179, Table 1</t>
+    </r>
+  </si>
+  <si>
+    <t>ARPA Veneto.  Laghi: concentrazione dei parametri di base – anni 2010-2019 (Open Data) sul portale dati.veneto.it: https://dati.veneto.it/content/laghi-concentrazione-dei-parametri-di-base-anni-2010-2019</t>
+  </si>
+  <si>
+    <t>ARPA Veneto.  Laghi: Livello Trofico per lo stato ecologico (LTLeco) nel periodo 2009-2024 (dataset CSV) sul portale Open Data Veneto: https://www.arpa.veneto.it/dati-ambientali/open-data/idrosfera/laghi/ltleco-livello-trofico-dei-laghi-per-lo-stato-ecologico</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Bevacqua, D., Andrello, M., Melià, P. A. C. O., Vincenzi, S., De Leo, G. A., &amp; Crivelli, A. J. (2011). Density-dependent and inter-specific interactions affecting European eel settlement in freshwater habitats. Hydrobiologia, 671(1), 259-265. Calculated from the information on canal length and width.</t>
+  </si>
+  <si>
+    <t>Vouvé, F., Buscail, R., Aubert, D., Labadie, P., Chevreuil, M., Canal, C., ... &amp; Biagianti-Risbourg, S. (2014). Bages-Sigean and Canet-St Nazaire lagoons (France): physico-chemical characteristics and contaminant concentrations (Cu, Cd, PCBs and PBDEs) as environmental quality of water and sediment. Environmental Science and Pollution Research, 21(4), 3005-3020.</t>
+  </si>
+  <si>
+    <t>Marchessaux, G., Nicolas, D., Crivelli, A., Befeld, S., Contournet, P., &amp; Thibault, D. (2020). Presence of the introduced ctenophore Mnemiopsis leidyi A. Agassiz, 1865 in a lagoon system within the River Rhône delta (southeast France). BioInvasions Records, 9(3), 471-481.</t>
+  </si>
+  <si>
+    <t>1,23,24,25,28,81</t>
+  </si>
+  <si>
+    <t>Garrido, M., Lafabrie, C., Torre, F., Fernandez, C., &amp; Pasqualini, V. (2013). Resilience and stability of Cymodocea nodosa seagrass meadows over the last four decades in a Mediterranean lagoon. Estuarine, Coastal and Shelf Science, 130, 89-98. Fig.6. Raw data 2000-2011 extracted from the figure using WebPlotDigitizer</t>
+  </si>
+  <si>
+    <t>Gianni, Areti &amp; Kehayias, George &amp; Zacharias, Ierotheos. (2012). Temporal and spatial distribution of physico-chemical parameters in an anoxic lagoon, Aitoliko, Greece. Journal of environmental biology / Academy of Environmental Biology, India. 33. 107-14. Table 2</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Patonai, K., Lanzoni, M., Castaldelli, G., Jordán, F., &amp; Gavioli, A. (2025). Eutrophication triggered changes in network structure and fluxes of the Comacchio Lagoon (Italy). </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PLOS ONE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 20(1), e0313416. https://doi.org/10.1371/journal.pone.0313416</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Table 1</t>
+    </r>
+  </si>
+  <si>
+    <t>Ounissi, M., Ziouch, O. R., &amp; Aounallah, O. (2014). Variability of the dissolved nutrient (N, P, Si) concentrations in the Bay of Annaba in relation to the inputs of the Seybouse and Mafragh estuaries. Marine pollution bulletin, 80(1-2), 234-244. Fig. 4, data digitized</t>
+  </si>
+  <si>
+    <t>Panfili, J., Darnaude, A. M., Lin, Y. J., Chevalley, M., Iizuka, Y., Tzeng, W. N., &amp; Crivelli, A. J. (2012). Habitat residence during continental life of the European eel Anguilla anguilla investigated using linear discriminant analysis applied to otolith Sr: Ca ratios. Aquatic Biology, 15(2), 175-185.</t>
+  </si>
+  <si>
+    <t>1,19,26,78,83</t>
+  </si>
+  <si>
+    <t>1,18,20,24,25,28,85</t>
+  </si>
+  <si>
+    <t>Leruste, A., Guilhaumon, F., De Wit, R., Malet, N., Collos, Y., &amp; Bec, B. (2019). Phytoplankton strategies to exploit nutrients in coastal lagoons with different eutrophication status during re-oligotrophication. Aquatic Microbial Ecology, 83(2), 131-146. Table 1</t>
+  </si>
+  <si>
+    <t>Pasqualini, V., Derolez, V., Garrido, M., Orsoni, V., Baldi, Y., Etourneau, S., ... &amp; Malet, N. (2017). Spatiotemporal dynamics of submerged macrophyte status and watershed exploitation in a Mediterranean coastal lagoon: Understanding critical factors in ecosystem degradation and restoration. Ecological Engineering, 102, 1-14.</t>
+  </si>
+  <si>
+    <t>1,23,24,25,28,87</t>
+  </si>
+  <si>
+    <t>1,18,20,24,25,28,84</t>
+  </si>
+  <si>
+    <t>1,18,20,24,25,28,80</t>
+  </si>
+  <si>
+    <t>Derolez, V., Soudant, D., Malet, N., Chiantella, C., Richard, M., Abadie, E., ... &amp; Bec, B. (2020). Two decades of oligotrophication: Evidence for a phytoplankton community shift in the coastal lagoon of Thau (Mediterranean Sea, France). Estuarine, Coastal and Shelf Science, 241, 106810.  Fig. 4a digitized</t>
+  </si>
+  <si>
+    <t>1,24,25,27,28,88</t>
+  </si>
+  <si>
+    <t>1,20,24,25,28,85</t>
+  </si>
+  <si>
+    <t>Gouze, E. (2008). Bilan de matière de l'étang de Berre: influence des apports des tributaires et des processus de régénération dans le maintien de l'eutrophisation (Doctoral dissertation, Aix-Marseille 2). Fig. III.38a digitized</t>
+  </si>
+  <si>
+    <t>1,20,24,25,28,89</t>
+  </si>
+  <si>
+    <t>SiteAcronym</t>
+  </si>
+  <si>
+    <t>DistanceGibraltar</t>
+  </si>
+  <si>
+    <t>Monitoring of eel in inland waters as part of the National Plan for Collection of Data in Fisheries of the Republic of Croatia (HRV DCF)</t>
+  </si>
+  <si>
+    <t>121, 13</t>
+  </si>
+  <si>
+    <t>various</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>lamiabendjedid@gmail.com</t>
+  </si>
+  <si>
+    <t>branko.glamuzina@unidu.hr</t>
+  </si>
+  <si>
+    <t>azzaelgan@yahoo.com</t>
+  </si>
+  <si>
+    <t>elsa.amilhat@univ-perp.fr</t>
+  </si>
+  <si>
+    <t>asapoun@inale.gr</t>
+  </si>
+  <si>
+    <t>chiara.leone@uniroma2.it</t>
+  </si>
+  <si>
+    <t>dragana.mi@ucg.ac.me</t>
+  </si>
+  <si>
+    <t>ba1fedec@uco.es</t>
+  </si>
+  <si>
+    <t>lluis.zamora@udg.edu</t>
+  </si>
+  <si>
+    <t>rachidtoujani2016@gmail.com</t>
+  </si>
+  <si>
+    <t>sozdilek@comu.edu.tr</t>
+  </si>
+  <si>
+    <t>Ciccotti, E. &amp; Morello, E.B. (eds). 2023. European eel in the Mediterranean Sea – Outcomes of the GFCM Research programme. Studies and Reviews No. 103 (General Fisheries Commission for the Mediterranean). Rome, FAO. https://doi.org/10.4060/cc7252en</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EPTB Lez (FILMED network)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PNR de la Narbonnaise en Méditerranée (FILMED network )</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Perpignan Agglomération (FILMED network)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maison de la Nature – Ville de Lattes (FILMED network)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EPTB Lez (FILMED network), Syndicat Mixte du Bassin de Thau</t>
+  </si>
+  <si>
+    <t>SMCG-Syndicat mixte de gestion de la camargue gardoise (FILMED network) </t>
+  </si>
+  <si>
+    <t>Communauté de communes La Domitienne (FILMED network) </t>
+  </si>
+  <si>
+    <t>SYMBO-Syndicat mixte du bassin de l'or (FILMED network)</t>
+  </si>
+  <si>
+    <t>Syndicat mixte RIVAGE (FILMED network)</t>
+  </si>
+  <si>
+    <t>Gipreb (FILMED network)</t>
+  </si>
+  <si>
+    <t>PNR de Camargue, SNPN-RNN de Camargue, CD13 (FILMED network)</t>
+  </si>
+  <si>
+    <t>leanderhoehne@gmx.net</t>
+  </si>
+  <si>
+    <t>Complex_Petite_Camargue, Complex_Vendres</t>
+  </si>
+  <si>
+    <t>Boutron, O., Grillas, P., Hilaire, S., Fontès, H., Luna-Laurent, E., &amp; Bec, B. (2022). Campagne de Surveillance 2021 de l’état DCE Des Lagunes Méditerranéennes Oligo-et Mésohalines Françaises Pour la Physico-Chimie, le Phytoplancton et les Macrophytes. Tour du Valat/Agence de l'Eau Rhône Méditerranée Corse. Figure B.3, digitized. https://medtrix.fr/wp-content/uploads/2019/09/DCE_Lagunes_Oligo_Meso_Haline_2015.pdf</t>
+  </si>
+  <si>
+    <t>Bec, B., Collos, Y., Souchu, P., Vaquer, A., Lautier, J., Fiandrino, A., ... &amp; Laugier, T. (2011). Distribution of picophytoplankton and nanophytoplankton along an anthropogenic eutrophication gradient in French Mediterranean coastal lagoons. Aquatic Microbial Ecology, 63(1), 29-45. Tab. 1. https://www.int-res.com/articles/ame2011/63/a063p029.pdf</t>
+  </si>
+  <si>
+    <t>NOTE: Multiple rows in the "Habitat_variables" sheet indicate measurements from distinct years, in which case these were averaged for further data analysis</t>
+  </si>
+  <si>
+    <t>For any questions on site- or country-specific data, a contact email address is given in column "X" of the Habitat_variables sheet. Please CC the first author, leanderhoehne@gmx.net, for coordination.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Djabourabi, A., Touati, H., Sehili, N., Boussadia, M. I., &amp; Bensouilah, M. (2017). </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Study of the physicochemical parameters of water and phytoplankton in Lake Tonga (wetland of the National Park of El Kala, North East of Algeria).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> International Journal of Biosciences, 11(3), 205‑218. https://doi.org/10.12692/ijb/11.3.205‑218. Figure 2A digitized</t>
+    </r>
+  </si>
+  <si>
+    <t>Souchu, P., Bec, B., Smith, V. H., Laugier, T., Fiandrino, A., Benau, L., ... &amp; Vaquer, A. (2010). Patterns in nutrient limitation and chlorophyll a along an anthropogenic eutrophication gradient in French Mediterranean coastal lagoons. Canadian Journal of Fisheries and Aquatic Sciences, 67(4), 743-753. https://archimer.ifremer.fr/doc/00003/11444/8002.pdf. Fig. 6 digitized</t>
+  </si>
+  <si>
+    <t>84,90</t>
+  </si>
+  <si>
+    <r>
+      <t>Ben Salem, F., Ben Said, O., Aissa, P., Mahmoudi, E., Monperrus, M., Grunberger, O., &amp; Duran, R. (2016). Pesticides in Ichkeul Lake–Bizerta Lagoon Watershed in Tunisia: use, occurrence, and effects on bacteria and free-living marine nematodes. </t>
     </r>
     <r>
       <rPr>
@@ -3248,274 +3523,10 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>GÜLÇİÇEK, O. (2018). Investigation of Water Quality of Akgöl Lake in the Göksu Delta. </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Advances in Ecological and Environmental Research</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 173-179, Table 1</t>
-    </r>
-  </si>
-  <si>
-    <t>ARPA Veneto.  Laghi: concentrazione dei parametri di base – anni 2010-2019 (Open Data) sul portale dati.veneto.it: https://dati.veneto.it/content/laghi-concentrazione-dei-parametri-di-base-anni-2010-2019</t>
-  </si>
-  <si>
-    <t>ARPA Veneto.  Laghi: Livello Trofico per lo stato ecologico (LTLeco) nel periodo 2009-2024 (dataset CSV) sul portale Open Data Veneto: https://www.arpa.veneto.it/dati-ambientali/open-data/idrosfera/laghi/ltleco-livello-trofico-dei-laghi-per-lo-stato-ecologico</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Djabourabi, A., Touati, H., Sehili, N., Boussadia, M. I., &amp; Bensouilah, M. (2017). </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Study of the physicochemical parameters of water and phytoplankton in Lake Tonga (wetland of the National Park of El Kala, North East of Algeria).</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> International Journal of Biosciences, 11(3), 205‑218. https://doi.org/10.12692/ijb/11.3.205‑218</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Figure 2A digitized</t>
-    </r>
-  </si>
-  <si>
-    <t>Bevacqua, D., Andrello, M., Melià, P. A. C. O., Vincenzi, S., De Leo, G. A., &amp; Crivelli, A. J. (2011). Density-dependent and inter-specific interactions affecting European eel settlement in freshwater habitats. Hydrobiologia, 671(1), 259-265. Calculated from the information on canal length and width.</t>
-  </si>
-  <si>
-    <t>Vouvé, F., Buscail, R., Aubert, D., Labadie, P., Chevreuil, M., Canal, C., ... &amp; Biagianti-Risbourg, S. (2014). Bages-Sigean and Canet-St Nazaire lagoons (France): physico-chemical characteristics and contaminant concentrations (Cu, Cd, PCBs and PBDEs) as environmental quality of water and sediment. Environmental Science and Pollution Research, 21(4), 3005-3020.</t>
-  </si>
-  <si>
-    <t>1,18,20,24,25,28,79</t>
-  </si>
-  <si>
-    <t>Marchessaux, G., Nicolas, D., Crivelli, A., Befeld, S., Contournet, P., &amp; Thibault, D. (2020). Presence of the introduced ctenophore Mnemiopsis leidyi A. Agassiz, 1865 in a lagoon system within the River Rhône delta (southeast France). BioInvasions Records, 9(3), 471-481.</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,80</t>
-  </si>
-  <si>
-    <t>1,23,24,25,28,81</t>
-  </si>
-  <si>
-    <t>Garrido, M., Lafabrie, C., Torre, F., Fernandez, C., &amp; Pasqualini, V. (2013). Resilience and stability of Cymodocea nodosa seagrass meadows over the last four decades in a Mediterranean lagoon. Estuarine, Coastal and Shelf Science, 130, 89-98. Fig.6. Raw data 2000-2011 extracted from the figure using WebPlotDigitizer</t>
-  </si>
-  <si>
-    <t>Gianni, Areti &amp; Kehayias, George &amp; Zacharias, Ierotheos. (2012). Temporal and spatial distribution of physico-chemical parameters in an anoxic lagoon, Aitoliko, Greece. Journal of environmental biology / Academy of Environmental Biology, India. 33. 107-14. Table 2</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Patonai, K., Lanzoni, M., Castaldelli, G., Jordán, F., &amp; Gavioli, A. (2025). Eutrophication triggered changes in network structure and fluxes of the Comacchio Lagoon (Italy). </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PLOS ONE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 20(1), e0313416. https://doi.org/10.1371/journal.pone.0313416</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Table 1</t>
-    </r>
-  </si>
-  <si>
-    <t>Ounissi, M., Ziouch, O. R., &amp; Aounallah, O. (2014). Variability of the dissolved nutrient (N, P, Si) concentrations in the Bay of Annaba in relation to the inputs of the Seybouse and Mafragh estuaries. Marine pollution bulletin, 80(1-2), 234-244. Fig. 4, data digitized</t>
-  </si>
-  <si>
-    <t>Panfili, J., Darnaude, A. M., Lin, Y. J., Chevalley, M., Iizuka, Y., Tzeng, W. N., &amp; Crivelli, A. J. (2012). Habitat residence during continental life of the European eel Anguilla anguilla investigated using linear discriminant analysis applied to otolith Sr: Ca ratios. Aquatic Biology, 15(2), 175-185.</t>
-  </si>
-  <si>
-    <t>1,19,26,78,83</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,79</t>
-  </si>
-  <si>
-    <t>Bec, B., Collos, Y., Souchu, P., Vaquer, A., Lautier, J., Fiandrino, A., ... &amp; Laugier, T. (2011). Distribution of picophytoplankton and nanophytoplankton along an anthropogenic eutrophication gradient in French Mediterranean coastal lagoons. Aquatic Microbial Ecology, 63(1), 29-45. Tab. 1</t>
-  </si>
-  <si>
-    <t>1,18,20,24,25,28,85</t>
-  </si>
-  <si>
-    <t>Leruste, A., Guilhaumon, F., De Wit, R., Malet, N., Collos, Y., &amp; Bec, B. (2019). Phytoplankton strategies to exploit nutrients in coastal lagoons with different eutrophication status during re-oligotrophication. Aquatic Microbial Ecology, 83(2), 131-146. Table 1</t>
-  </si>
-  <si>
-    <t>Boutron, O., Grillas, P., Hilaire, S., Fontès, H., Luna-Laurent, E., &amp; Bec, B. (2022). Campagne de Surveillance 2021 de l’état DCE Des Lagunes Méditerranéennes Oligo-et Mésohalines Françaises Pour la Physico-Chimie, le Phytoplancton et les Macrophytes. Tour du Valat/Agence de l'Eau Rhône Méditerranée Corse. Figure B.3, digitized</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,84,86</t>
-  </si>
-  <si>
-    <t>Pasqualini, V., Derolez, V., Garrido, M., Orsoni, V., Baldi, Y., Etourneau, S., ... &amp; Malet, N. (2017). Spatiotemporal dynamics of submerged macrophyte status and watershed exploitation in a Mediterranean coastal lagoon: Understanding critical factors in ecosystem degradation and restoration. Ecological Engineering, 102, 1-14.</t>
-  </si>
-  <si>
-    <t>1,23,24,25,28,87</t>
-  </si>
-  <si>
-    <t>1,18,20,24,25,28,84</t>
-  </si>
-  <si>
-    <t>1,18,20,24,25,28,80</t>
-  </si>
-  <si>
-    <t>Derolez, V., Soudant, D., Malet, N., Chiantella, C., Richard, M., Abadie, E., ... &amp; Bec, B. (2020). Two decades of oligotrophication: Evidence for a phytoplankton community shift in the coastal lagoon of Thau (Mediterranean Sea, France). Estuarine, Coastal and Shelf Science, 241, 106810.  Fig. 4a digitized</t>
-  </si>
-  <si>
-    <t>1,24,25,27,28,88</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,85</t>
-  </si>
-  <si>
-    <t>Gouze, E. (2008). Bilan de matière de l'étang de Berre: influence des apports des tributaires et des processus de régénération dans le maintien de l'eutrophisation (Doctoral dissertation, Aix-Marseille 2). Fig. III.38a digitized</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,89</t>
-  </si>
-  <si>
-    <t>Souchu, P., Bec, B., Smith, V. H., Laugier, T., Fiandrino, A., Benau, L., ... &amp; Vaquer, A. (2010). Patterns in nutrient limitation and chlorophyll a along an anthropogenic eutrophication gradient in French Mediterranean coastal lagoons. Canadian Journal of Fisheries and Aquatic Sciences, 67(4), 743-753. Fig. 6 digitized</t>
-  </si>
-  <si>
-    <t>1,20,24,25,28,84,90</t>
-  </si>
-  <si>
-    <t>SiteAcronym</t>
-  </si>
-  <si>
-    <t>DistanceGibraltar</t>
-  </si>
-  <si>
-    <t>Monitoring of eel in inland waters as part of the National Plan for Collection of Data in Fisheries of the Republic of Croatia (HRV DCF)</t>
-  </si>
-  <si>
-    <t>121, 13</t>
-  </si>
-  <si>
-    <t>various</t>
-  </si>
-  <si>
-    <t>Contact</t>
-  </si>
-  <si>
-    <t>lamiabendjedid@gmail.com</t>
-  </si>
-  <si>
-    <t>branko.glamuzina@unidu.hr</t>
-  </si>
-  <si>
-    <t>azzaelgan@yahoo.com</t>
-  </si>
-  <si>
-    <t>elsa.amilhat@univ-perp.fr</t>
-  </si>
-  <si>
-    <t>asapoun@inale.gr</t>
-  </si>
-  <si>
-    <t>chiara.leone@uniroma2.it</t>
-  </si>
-  <si>
-    <t>dragana.mi@ucg.ac.me</t>
-  </si>
-  <si>
-    <t>ba1fedec@uco.es</t>
-  </si>
-  <si>
-    <t>lluis.zamora@udg.edu</t>
-  </si>
-  <si>
-    <t>rachidtoujani2016@gmail.com</t>
-  </si>
-  <si>
-    <t>sozdilek@comu.edu.tr</t>
+    <t>1,70,76</t>
+  </si>
+  <si>
+    <t>1,68,77</t>
   </si>
 </sst>
 </file>
@@ -3689,7 +3700,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -3770,6 +3781,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -4077,7 +4094,7 @@
     <col min="19" max="19" width="20.46484375" style="1" customWidth="1"/>
     <col min="20" max="20" width="33" style="1" customWidth="1"/>
     <col min="21" max="22" width="25.86328125" style="1" customWidth="1"/>
-    <col min="23" max="23" width="15.53125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.06640625" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
@@ -4121,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>164</v>
@@ -4181,13 +4198,13 @@
         <v>52</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="X2" s="15" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4258,10 +4275,10 @@
         <v>1325058.5762481689</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="X3" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4332,10 +4349,10 @@
         <v>1325058.5762481689</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="X4" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4406,10 +4423,10 @@
         <v>1325058.5762481689</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="X5" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4480,10 +4497,10 @@
         <v>1325058.5762481689</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="X6" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4554,10 +4571,10 @@
         <v>1325058.5762481689</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="X7" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4627,11 +4644,11 @@
       <c r="V8" s="1">
         <v>1331104.3170471191</v>
       </c>
-      <c r="W8" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="X8" s="27" t="s">
-        <v>330</v>
+      <c r="W8" s="1">
+        <v>5</v>
+      </c>
+      <c r="X8" s="28" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4702,10 +4719,10 @@
         <v>1331104.3170471191</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="X9" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4776,10 +4793,10 @@
         <v>1331104.3170471191</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="X10" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4850,10 +4867,10 @@
         <v>1331104.3170471191</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="X11" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4924,10 +4941,10 @@
         <v>1331104.3170471191</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="X12" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -4998,10 +5015,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X13" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5072,10 +5089,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X14" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5146,10 +5163,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X15" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5220,10 +5237,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X16" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5294,10 +5311,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X17" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5368,10 +5385,10 @@
         <v>1314655.8920135498</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X18" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5442,10 +5459,10 @@
         <v>1285588.6951293945</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="X19" s="27" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.45">
@@ -5507,7 +5524,7 @@
         <v>121</v>
       </c>
       <c r="X20" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.45">
@@ -5569,7 +5586,7 @@
         <v>121</v>
       </c>
       <c r="X21" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.45">
@@ -5631,7 +5648,7 @@
         <v>121</v>
       </c>
       <c r="X22" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -5692,10 +5709,10 @@
         <v>2884204.3825531006</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="X23" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.45">
@@ -5757,7 +5774,7 @@
         <v>121</v>
       </c>
       <c r="X24" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.45">
@@ -5819,7 +5836,7 @@
         <v>121</v>
       </c>
       <c r="X25" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.45">
@@ -5881,7 +5898,7 @@
         <v>121</v>
       </c>
       <c r="X26" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.45">
@@ -5943,7 +5960,7 @@
         <v>121</v>
       </c>
       <c r="X27" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.45">
@@ -6005,7 +6022,7 @@
         <v>121</v>
       </c>
       <c r="X28" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.45">
@@ -6067,7 +6084,7 @@
         <v>121</v>
       </c>
       <c r="X29" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.45">
@@ -6129,7 +6146,7 @@
         <v>121</v>
       </c>
       <c r="X30" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6200,10 +6217,10 @@
         <v>3780197.4512481689</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="X31" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
     </row>
     <row r="32" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6274,10 +6291,10 @@
         <v>3643490.0868530273</v>
       </c>
       <c r="W32" s="1" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="X32" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6348,10 +6365,10 @@
         <v>3872223.5192260742</v>
       </c>
       <c r="W33" s="1" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="X33" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
     </row>
     <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6408,7 +6425,7 @@
         <v>1</v>
       </c>
       <c r="X34" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6464,7 +6481,7 @@
         <v>1</v>
       </c>
       <c r="X35" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6535,10 +6552,10 @@
         <v>1326723.4623718262</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="X36" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6609,10 +6626,10 @@
         <v>1265951.7396392822</v>
       </c>
       <c r="W37" s="1" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="X37" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6682,11 +6699,11 @@
       <c r="V38" s="1">
         <v>1265951.7396392822</v>
       </c>
-      <c r="W38" s="1" t="s">
-        <v>297</v>
+      <c r="W38" s="1">
+        <v>79</v>
       </c>
       <c r="X38" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6757,10 +6774,10 @@
         <v>1336349.1169891357</v>
       </c>
       <c r="W39" s="1" t="s">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="X39" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6831,10 +6848,10 @@
         <v>1216347.9565429688</v>
       </c>
       <c r="W40" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X40" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6904,11 +6921,11 @@
       <c r="V41" s="1">
         <v>1216347.9565429688</v>
       </c>
-      <c r="W41" s="1" t="s">
-        <v>307</v>
+      <c r="W41" s="1">
+        <v>79</v>
       </c>
       <c r="X41" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="42" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -6979,10 +6996,10 @@
         <v>1261115.409072876</v>
       </c>
       <c r="W42" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X42" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="43" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7053,10 +7070,10 @@
         <v>1261115.409072876</v>
       </c>
       <c r="W43" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X43" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="44" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7127,10 +7144,10 @@
         <v>1261115.409072876</v>
       </c>
       <c r="W44" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X44" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="45" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7201,10 +7218,10 @@
         <v>1261115.409072876</v>
       </c>
       <c r="W45" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X45" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="46" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7275,10 +7292,10 @@
         <v>1261115.409072876</v>
       </c>
       <c r="W46" s="1" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="X46" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="47" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7349,10 +7366,10 @@
         <v>1327891.767791748</v>
       </c>
       <c r="W47" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X47" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="48" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7422,11 +7439,11 @@
       <c r="V48" s="1">
         <v>1327891.767791748</v>
       </c>
-      <c r="W48" s="1" t="s">
-        <v>323</v>
+      <c r="W48" s="29" t="s">
+        <v>346</v>
       </c>
       <c r="X48" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="49" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7497,10 +7514,10 @@
         <v>1327891.767791748</v>
       </c>
       <c r="W49" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X49" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="50" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7571,10 +7588,10 @@
         <v>1327891.767791748</v>
       </c>
       <c r="W50" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X50" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="51" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7644,11 +7661,11 @@
       <c r="V51" s="1">
         <v>1327891.767791748</v>
       </c>
-      <c r="W51" s="1" t="s">
-        <v>323</v>
+      <c r="W51" s="29" t="s">
+        <v>346</v>
       </c>
       <c r="X51" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="52" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7662,7 +7679,7 @@
         <v>118</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E52" s="17">
         <v>4.1469079999999998</v>
@@ -7719,10 +7736,10 @@
         <v>1327891.767791748</v>
       </c>
       <c r="W52" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X52" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="53" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7736,7 +7753,7 @@
         <v>118</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E53" s="17">
         <v>4.013388</v>
@@ -7793,10 +7810,10 @@
         <v>1327891.767791748</v>
       </c>
       <c r="W53" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X53" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="54" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7867,10 +7884,10 @@
         <v>1328172.6247558594</v>
       </c>
       <c r="W54" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X54" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -7940,11 +7957,11 @@
       <c r="V55" s="1">
         <v>1328172.6247558594</v>
       </c>
-      <c r="W55" s="1" t="s">
-        <v>299</v>
+      <c r="W55" s="1">
+        <v>80</v>
       </c>
       <c r="X55" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="56" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8015,10 +8032,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W56" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="X56" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="57" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8089,10 +8106,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W57" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="X57" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="58" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8163,10 +8180,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W58" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X58" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="59" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8236,11 +8253,11 @@
       <c r="V59" s="1">
         <v>1273657.0374450684</v>
       </c>
-      <c r="W59" s="1" t="s">
-        <v>312</v>
+      <c r="W59" s="1">
+        <v>84.86</v>
       </c>
       <c r="X59" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="60" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8254,7 +8271,7 @@
         <v>125</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E60" s="17">
         <v>3.405948</v>
@@ -8311,10 +8328,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W60" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="X60" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="61" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8328,7 +8345,7 @@
         <v>126</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E61" s="17">
         <v>3.3024279999999999</v>
@@ -8385,10 +8402,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W61" s="1" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="X61" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="62" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8402,7 +8419,7 @@
         <v>126</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E62" s="17">
         <v>3.0472969999999999</v>
@@ -8459,10 +8476,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W62" s="1" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="X62" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="63" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8476,7 +8493,7 @@
         <v>125</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E63" s="17">
         <v>3.2225000000000001</v>
@@ -8533,10 +8550,10 @@
         <v>1273657.0374450684</v>
       </c>
       <c r="W63" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="X63" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="64" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8607,10 +8624,10 @@
         <v>1656125.4413757324</v>
       </c>
       <c r="W64" s="1" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="X64" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="65" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8681,10 +8698,10 @@
         <v>1656125.4413757324</v>
       </c>
       <c r="W65" s="1" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="X65" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="66" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8755,10 +8772,10 @@
         <v>1656125.4413757324</v>
       </c>
       <c r="W66" s="1" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="X66" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="67" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8829,10 +8846,10 @@
         <v>1325944.5123901367</v>
       </c>
       <c r="W67" s="1" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
       <c r="X67" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="68" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8903,10 +8920,10 @@
         <v>1243945.1788024902</v>
       </c>
       <c r="W68" s="1" t="s">
-        <v>316</v>
+        <v>303</v>
       </c>
       <c r="X68" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="69" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -8977,10 +8994,10 @@
         <v>1295319.2137145996</v>
       </c>
       <c r="W69" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="X69" t="s">
         <v>318</v>
-      </c>
-      <c r="X69" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9051,10 +9068,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W70" s="1" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="X70" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="71" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9125,10 +9142,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W71" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X71" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="72" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9199,10 +9216,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W72" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X72" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="73" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9273,10 +9290,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W73" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X73" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="74" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9347,10 +9364,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W74" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X74" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="75" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9421,10 +9438,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W75" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X75" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="76" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9495,10 +9512,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W76" s="1" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="X76" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="77" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9569,10 +9586,10 @@
         <v>1315297.4694824219</v>
       </c>
       <c r="W77" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X77" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
     </row>
     <row r="78" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9643,10 +9660,10 @@
         <v>3262408.4235839844</v>
       </c>
       <c r="W78" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="X78" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
     </row>
     <row r="79" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9717,10 +9734,10 @@
         <v>2559583.9927368164</v>
       </c>
       <c r="W79" s="1" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="X79" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
     </row>
     <row r="80" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9791,10 +9808,10 @@
         <v>2537136.3298339844</v>
       </c>
       <c r="W80" s="1" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="X80" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
     </row>
     <row r="81" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9868,7 +9885,7 @@
         <v>1</v>
       </c>
       <c r="X81" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="82" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -9942,7 +9959,7 @@
         <v>1</v>
       </c>
       <c r="X82" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="83" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10013,10 +10030,10 @@
         <v>3232493.6495361328</v>
       </c>
       <c r="W83" s="1" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="X83" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="84" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10024,10 +10041,10 @@
         <v>63</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>24</v>
@@ -10087,10 +10104,10 @@
         <v>1824624.9945220947</v>
       </c>
       <c r="W84" s="1" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="X84" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="85" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10161,10 +10178,10 @@
         <v>1826019.0267486572</v>
       </c>
       <c r="W85" s="1" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="X85" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="86" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10235,10 +10252,10 @@
         <v>1846828.1826934814</v>
       </c>
       <c r="W86" s="1" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="X86" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="87" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10246,10 +10263,10 @@
         <v>63</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>34</v>
@@ -10309,10 +10326,10 @@
         <v>3184787.2149200439</v>
       </c>
       <c r="W87" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="X87" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="88" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10320,10 +10337,10 @@
         <v>63</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>34</v>
@@ -10383,10 +10400,10 @@
         <v>3221879.1607055664</v>
       </c>
       <c r="W88" s="1" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="X88" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="89" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10457,10 +10474,10 @@
         <v>3182562.3193664551</v>
       </c>
       <c r="W89" s="1" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="X89" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="90" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10531,10 +10548,10 @@
         <v>3182562.3193664551</v>
       </c>
       <c r="W90" s="1" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="X90" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="91" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10605,10 +10622,10 @@
         <v>1798583.0234985352</v>
       </c>
       <c r="W91" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="X91" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="92" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10616,10 +10633,10 @@
         <v>63</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>34</v>
@@ -10679,10 +10696,10 @@
         <v>2781070.9394378662</v>
       </c>
       <c r="W92" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="X92" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="93" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10690,10 +10707,10 @@
         <v>63</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>34</v>
@@ -10753,10 +10770,10 @@
         <v>2754117.4776916504</v>
       </c>
       <c r="W93" s="1" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="X93" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="94" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10827,10 +10844,10 @@
         <v>1883372.305557251</v>
       </c>
       <c r="W94" s="1" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="X94" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="95" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10838,10 +10855,10 @@
         <v>63</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>34</v>
@@ -10901,10 +10918,10 @@
         <v>1451476.6793670654</v>
       </c>
       <c r="W95" s="1" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="X95" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="96" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -10912,10 +10929,10 @@
         <v>63</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>34</v>
@@ -10975,10 +10992,10 @@
         <v>1411840.9035186768</v>
       </c>
       <c r="W96" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="X96" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="97" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11049,10 +11066,10 @@
         <v>3222141.7445678711</v>
       </c>
       <c r="W97" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="X97" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="98" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11123,10 +11140,10 @@
         <v>1845988.7758483887</v>
       </c>
       <c r="W98" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="X98" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="99" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11188,10 +11205,10 @@
         <v>2646019.1369781494</v>
       </c>
       <c r="W99" s="1" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="X99" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
     </row>
     <row r="100" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11262,10 +11279,10 @@
         <v>1097854.6567993164</v>
       </c>
       <c r="W100" s="1" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="X100" t="s">
-        <v>338</v>
+        <v>323</v>
       </c>
     </row>
     <row r="101" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11336,10 +11353,10 @@
         <v>75401.811233520508</v>
       </c>
       <c r="W101" s="1" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="X101" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
     </row>
     <row r="102" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11410,10 +11427,10 @@
         <v>1473707.8613433838</v>
       </c>
       <c r="W102" s="1" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="X102" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
     <row r="103" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11484,10 +11501,10 @@
         <v>1473707.8613433838</v>
       </c>
       <c r="W103" s="1" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="X103" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
     <row r="104" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11561,7 +11578,7 @@
         <v>1</v>
       </c>
       <c r="X104" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
     <row r="105" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11635,7 +11652,7 @@
         <v>1</v>
       </c>
       <c r="X105" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
     <row r="106" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11706,10 +11723,10 @@
         <v>3249104.3733215332</v>
       </c>
       <c r="W106" s="1" t="s">
-        <v>252</v>
+        <v>348</v>
       </c>
       <c r="X106" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
     <row r="107" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11779,11 +11796,11 @@
       <c r="V107" s="1">
         <v>3249104.3733215332</v>
       </c>
-      <c r="W107" s="1" t="s">
-        <v>252</v>
+      <c r="W107" s="1">
+        <v>71</v>
       </c>
       <c r="X107" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="108" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11854,10 +11871,10 @@
         <v>3122441.9502258301</v>
       </c>
       <c r="W108" s="1" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="X108" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
     <row r="109" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -11928,10 +11945,10 @@
         <v>3701580.7314453125</v>
       </c>
       <c r="W109" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="X109" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
     <row r="110" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -12002,10 +12019,10 @@
         <v>3184749.3204193115</v>
       </c>
       <c r="W110" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="X110" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
     <row r="111" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -12076,10 +12093,10 @@
         <v>3871417.8141479492</v>
       </c>
       <c r="W111" s="1" t="s">
-        <v>250</v>
+        <v>349</v>
       </c>
       <c r="X111" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
     <row r="112" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -12150,10 +12167,10 @@
         <v>3871417.8141479492</v>
       </c>
       <c r="W112" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="X112" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -12176,10 +12193,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF334FA7-C150-4F6F-A6B2-7716EC54D70C}">
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18.53125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="18.53125" style="7"/>
+    <col min="1" max="1" width="18.53125" style="7"/>
+    <col min="2" max="2" width="37.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="60.19921875" style="7" customWidth="1"/>
     <col min="4" max="4" width="18.53125" style="26"/>
     <col min="5" max="16384" width="18.53125" style="7"/>
@@ -12201,13 +12219,13 @@
     </row>
     <row r="2" spans="1:4" s="14" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="9" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>211</v>
+        <v>326</v>
       </c>
       <c r="D2" s="24">
         <v>1</v>
@@ -12221,7 +12239,7 @@
         <v>92</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D3" s="25">
         <v>2</v>
@@ -12235,7 +12253,7 @@
         <v>80</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D4" s="25">
         <v>2</v>
@@ -12249,7 +12267,7 @@
         <v>78</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D5" s="25">
         <v>2</v>
@@ -12263,7 +12281,7 @@
         <v>78</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D6" s="25">
         <v>3</v>
@@ -12277,7 +12295,7 @@
         <v>80</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D7" s="25">
         <v>4</v>
@@ -12291,7 +12309,7 @@
         <v>80</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>294</v>
+        <v>344</v>
       </c>
       <c r="D8" s="25">
         <v>5</v>
@@ -12305,7 +12323,7 @@
         <v>92</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D9" s="25">
         <v>6</v>
@@ -12319,7 +12337,7 @@
         <v>80</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D10" s="25">
         <v>7</v>
@@ -12333,7 +12351,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D11" s="25">
         <v>7</v>
@@ -12347,24 +12365,24 @@
         <v>92</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D12" s="25">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="8" t="s">
         <v>57</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>304</v>
+      <c r="C13" s="6" t="s">
+        <v>260</v>
       </c>
       <c r="D13" s="25">
-        <v>82</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -12372,13 +12390,13 @@
         <v>57</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>265</v>
+        <v>78</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>179</v>
       </c>
       <c r="D14" s="25">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
@@ -12389,24 +12407,24 @@
         <v>78</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D15" s="25">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>78</v>
+        <v>313</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>182</v>
+        <v>311</v>
       </c>
       <c r="D16" s="25">
-        <v>11</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
@@ -12414,13 +12432,13 @@
         <v>35</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>326</v>
+        <v>38</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>261</v>
       </c>
       <c r="D17" s="25">
-        <v>121</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
@@ -12428,13 +12446,13 @@
         <v>35</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D18" s="25">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
@@ -12442,13 +12460,13 @@
         <v>35</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D19" s="25">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -12456,10 +12474,10 @@
         <v>35</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D20" s="25">
         <v>14</v>
@@ -12467,16 +12485,16 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="8" t="s">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D21" s="25">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
@@ -12484,13 +12502,13 @@
         <v>95</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D22" s="25">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
@@ -12498,27 +12516,27 @@
         <v>95</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="D23" s="25">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24" s="8" t="s">
-        <v>95</v>
+      <c r="A24" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>254</v>
+        <v>102</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>167</v>
       </c>
       <c r="D24" s="25">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
@@ -12526,7 +12544,7 @@
         <v>48</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>167</v>
@@ -12540,10 +12558,10 @@
         <v>48</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D26" s="25">
         <v>18</v>
@@ -12554,10 +12572,10 @@
         <v>48</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D27" s="25">
         <v>18</v>
@@ -12568,13 +12586,13 @@
         <v>48</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D28" s="25">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
@@ -12582,13 +12600,13 @@
         <v>48</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>308</v>
+        <v>168</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>327</v>
       </c>
       <c r="D29" s="25">
-        <v>84</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
@@ -12596,13 +12614,13 @@
         <v>48</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>295</v>
+        <v>328</v>
       </c>
       <c r="D30" s="25">
-        <v>78</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
@@ -12610,13 +12628,13 @@
         <v>48</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>171</v>
+        <v>328</v>
       </c>
       <c r="D31" s="25">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
@@ -12624,13 +12642,13 @@
         <v>48</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>311</v>
+        <v>328</v>
       </c>
       <c r="D32" s="25">
-        <v>86</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
@@ -12638,13 +12656,13 @@
         <v>48</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="D33" s="25">
-        <v>88</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
@@ -12652,10 +12670,10 @@
         <v>48</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>168</v>
+        <v>112</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>172</v>
+        <v>328</v>
       </c>
       <c r="D34" s="25">
         <v>20</v>
@@ -12666,10 +12684,10 @@
         <v>48</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>172</v>
+        <v>328</v>
       </c>
       <c r="D35" s="25">
         <v>20</v>
@@ -12680,10 +12698,10 @@
         <v>48</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>209</v>
+        <v>328</v>
       </c>
       <c r="D36" s="25">
         <v>20</v>
@@ -12694,10 +12712,10 @@
         <v>48</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>172</v>
+        <v>328</v>
       </c>
       <c r="D37" s="25">
         <v>20</v>
@@ -12708,10 +12726,10 @@
         <v>48</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>172</v>
+        <v>330</v>
       </c>
       <c r="D38" s="25">
         <v>20</v>
@@ -12722,10 +12740,10 @@
         <v>48</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>172</v>
+        <v>327</v>
       </c>
       <c r="D39" s="25">
         <v>20</v>
@@ -12736,10 +12754,10 @@
         <v>48</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>110</v>
+        <v>139</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>172</v>
+        <v>327</v>
       </c>
       <c r="D40" s="25">
         <v>20</v>
@@ -12750,10 +12768,10 @@
         <v>48</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>172</v>
+        <v>327</v>
       </c>
       <c r="D41" s="25">
         <v>20</v>
@@ -12764,10 +12782,10 @@
         <v>48</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>172</v>
+        <v>331</v>
       </c>
       <c r="D42" s="25">
         <v>20</v>
@@ -12778,10 +12796,10 @@
         <v>48</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>172</v>
+        <v>331</v>
       </c>
       <c r="D43" s="25">
         <v>20</v>
@@ -12792,10 +12810,10 @@
         <v>48</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>172</v>
+        <v>331</v>
       </c>
       <c r="D44" s="25">
         <v>20</v>
@@ -12806,10 +12824,10 @@
         <v>48</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>172</v>
+        <v>331</v>
       </c>
       <c r="D45" s="25">
         <v>20</v>
@@ -12820,10 +12838,10 @@
         <v>48</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>172</v>
+        <v>332</v>
       </c>
       <c r="D46" s="25">
         <v>20</v>
@@ -12834,10 +12852,10 @@
         <v>48</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>172</v>
+        <v>332</v>
       </c>
       <c r="D47" s="25">
         <v>20</v>
@@ -12848,10 +12866,10 @@
         <v>48</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>172</v>
+        <v>332</v>
       </c>
       <c r="D48" s="25">
         <v>20</v>
@@ -12862,7 +12880,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>172</v>
@@ -12876,10 +12894,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>172</v>
+        <v>337</v>
       </c>
       <c r="D50" s="25">
         <v>20</v>
@@ -12890,10 +12908,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>172</v>
+        <v>333</v>
       </c>
       <c r="D51" s="25">
         <v>20</v>
@@ -12904,10 +12922,10 @@
         <v>48</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>172</v>
+        <v>334</v>
       </c>
       <c r="D52" s="25">
         <v>20</v>
@@ -12918,10 +12936,10 @@
         <v>48</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>172</v>
+        <v>335</v>
       </c>
       <c r="D53" s="25">
         <v>20</v>
@@ -12932,10 +12950,10 @@
         <v>48</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>172</v>
+        <v>336</v>
       </c>
       <c r="D54" s="25">
         <v>20</v>
@@ -12946,13 +12964,13 @@
         <v>48</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>173</v>
+        <v>126</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>172</v>
       </c>
       <c r="D55" s="25">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.45">
@@ -12960,13 +12978,13 @@
         <v>48</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D56" s="25">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.45">
@@ -12974,41 +12992,41 @@
         <v>48</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D57" s="25">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A58" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B58" s="8" t="s">
-        <v>131</v>
+      <c r="B58" s="5" t="s">
+        <v>166</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>172</v>
+        <v>205</v>
       </c>
       <c r="D58" s="25">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A59" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B59" s="8" t="s">
-        <v>104</v>
+      <c r="B59" s="5" t="s">
+        <v>166</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>169</v>
+        <v>204</v>
       </c>
       <c r="D59" s="25">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.45">
@@ -13016,13 +13034,13 @@
         <v>48</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>301</v>
+        <v>250</v>
       </c>
       <c r="D60" s="25">
-        <v>81</v>
+        <v>26</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.45">
@@ -13030,265 +13048,265 @@
         <v>48</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>320</v>
+        <v>174</v>
       </c>
       <c r="D61" s="25">
-        <v>89</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A62" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B62" s="8" t="s">
-        <v>107</v>
+      <c r="B62" s="5" t="s">
+        <v>166</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>310</v>
+        <v>206</v>
       </c>
       <c r="D62" s="25">
-        <v>85</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A63" s="5" t="s">
-        <v>48</v>
+      <c r="A63" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>174</v>
+        <v>152</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>266</v>
       </c>
       <c r="D63" s="25">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A64" s="5" t="s">
-        <v>48</v>
+      <c r="A64" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>298</v>
+        <v>152</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>267</v>
       </c>
       <c r="D64" s="25">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A65" s="5" t="s">
-        <v>48</v>
+      <c r="A65" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>170</v>
+        <v>293</v>
       </c>
       <c r="D65" s="25">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A66" s="5" t="s">
-        <v>48</v>
+      <c r="A66" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>170</v>
+        <v>148</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>184</v>
       </c>
       <c r="D66" s="25">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A67" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>166</v>
+      <c r="A67" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>199</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>207</v>
+        <v>251</v>
       </c>
       <c r="D67" s="25">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A68" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>166</v>
+      <c r="A68" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="D68" s="25">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A69" s="5" t="s">
-        <v>48</v>
+      <c r="A69" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>133</v>
+        <v>199</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>305</v>
+        <v>280</v>
       </c>
       <c r="D69" s="25">
-        <v>83</v>
+        <v>35</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A70" s="5" t="s">
-        <v>48</v>
+      <c r="A70" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>313</v>
+        <v>227</v>
       </c>
       <c r="D70" s="25">
-        <v>87</v>
+        <v>36</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A71" s="5" t="s">
-        <v>48</v>
+      <c r="A71" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>133</v>
+        <v>191</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D71" s="25">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A72" s="5" t="s">
-        <v>48</v>
+      <c r="A72" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>132</v>
+        <v>192</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>176</v>
+        <v>252</v>
       </c>
       <c r="D72" s="25">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A73" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B73" s="5" t="s">
-        <v>166</v>
+      <c r="A73" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>190</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="D73" s="25">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A74" s="5" t="s">
-        <v>48</v>
+      <c r="A74" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>322</v>
+        <v>253</v>
       </c>
       <c r="D74" s="25">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A75" s="5" t="s">
-        <v>48</v>
+      <c r="A75" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>102</v>
+        <v>196</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="D75" s="25">
-        <v>79</v>
+        <v>40</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A76" s="8" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>271</v>
+        <v>154</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>226</v>
       </c>
       <c r="D76" s="25">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A77" s="8" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>272</v>
+        <v>198</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>255</v>
       </c>
       <c r="D77" s="25">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A78" s="8" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>150</v>
+        <v>81</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="D78" s="25">
-        <v>31</v>
+        <v>43</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A79" s="8" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="C79" s="8" t="s">
-        <v>186</v>
+        <v>81</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="D79" s="25">
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.45">
@@ -13296,13 +13314,13 @@
         <v>63</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="C80" s="5" t="s">
-        <v>231</v>
+        <v>199</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>256</v>
       </c>
       <c r="D80" s="25">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.45">
@@ -13310,13 +13328,13 @@
         <v>63</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>256</v>
+        <v>194</v>
       </c>
       <c r="D81" s="25">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.45">
@@ -13324,13 +13342,13 @@
         <v>63</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>155</v>
+        <v>187</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>228</v>
+        <v>188</v>
       </c>
       <c r="D82" s="25">
-        <v>34</v>
+        <v>46</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.45">
@@ -13338,13 +13356,13 @@
         <v>63</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>285</v>
+        <v>188</v>
       </c>
       <c r="D83" s="25">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.45">
@@ -13352,13 +13370,13 @@
         <v>63</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>257</v>
+        <v>188</v>
       </c>
       <c r="D84" s="25">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.45">
@@ -13366,13 +13384,13 @@
         <v>63</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>257</v>
+        <v>188</v>
       </c>
       <c r="D85" s="25">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.45">
@@ -13380,13 +13398,13 @@
         <v>63</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>260</v>
+        <v>190</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>268</v>
       </c>
       <c r="D86" s="25">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.45">
@@ -13394,13 +13412,13 @@
         <v>63</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>81</v>
+        <v>193</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>291</v>
+        <v>195</v>
       </c>
       <c r="D87" s="25">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.45">
@@ -13408,13 +13426,13 @@
         <v>63</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>292</v>
+        <v>192</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>269</v>
       </c>
       <c r="D88" s="25">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.45">
@@ -13422,13 +13440,13 @@
         <v>63</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>229</v>
+        <v>191</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>269</v>
       </c>
       <c r="D89" s="25">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.45">
@@ -13436,13 +13454,13 @@
         <v>63</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>258</v>
+        <v>186</v>
       </c>
       <c r="D90" s="25">
-        <v>39</v>
+        <v>51</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.45">
@@ -13450,13 +13468,13 @@
         <v>63</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>198</v>
+        <v>153</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>259</v>
+        <v>294</v>
       </c>
       <c r="D91" s="25">
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.45">
@@ -13464,13 +13482,13 @@
         <v>63</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>230</v>
+        <v>198</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>270</v>
       </c>
       <c r="D92" s="25">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.45">
@@ -13478,13 +13496,13 @@
         <v>63</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>261</v>
+        <v>196</v>
+      </c>
+      <c r="C93" s="5" t="s">
+        <v>197</v>
       </c>
       <c r="D93" s="25">
-        <v>45</v>
+        <v>54</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.45">
@@ -13492,13 +13510,13 @@
         <v>63</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="D94" s="25">
-        <v>46</v>
+        <v>55</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.45">
@@ -13506,13 +13524,13 @@
         <v>63</v>
       </c>
       <c r="B95" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C95" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C95" s="5" t="s">
-        <v>190</v>
-      </c>
       <c r="D95" s="25">
-        <v>46</v>
+        <v>55</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.45">
@@ -13520,13 +13538,13 @@
         <v>63</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>192</v>
+        <v>154</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D96" s="25">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.45">
@@ -13534,13 +13552,13 @@
         <v>63</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D97" s="25">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.45">
@@ -13548,13 +13566,13 @@
         <v>63</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D98" s="25">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.45">
@@ -13562,13 +13580,13 @@
         <v>63</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>192</v>
+        <v>154</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D99" s="25">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.45">
@@ -13576,13 +13594,13 @@
         <v>63</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>197</v>
+        <v>192</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>271</v>
       </c>
       <c r="D100" s="25">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.45">
@@ -13590,13 +13608,13 @@
         <v>63</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>194</v>
+        <v>86</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
       <c r="D101" s="25">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.45">
@@ -13604,506 +13622,494 @@
         <v>63</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>193</v>
+        <v>87</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
       <c r="D102" s="25">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A103" s="8" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="C103" s="5" t="s">
-        <v>188</v>
+        <v>29</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>281</v>
       </c>
       <c r="D103" s="25">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A104" s="8" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>153</v>
+        <v>29</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>303</v>
+        <v>282</v>
       </c>
       <c r="D104" s="25">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A105" s="8" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>200</v>
+        <v>29</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D105" s="25">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A106" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>198</v>
+        <v>70</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D106" s="25">
-        <v>54</v>
+        <v>61</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A107" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>189</v>
+        <v>70</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="D107" s="25">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A108" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D108" s="25">
         <v>63</v>
-      </c>
-      <c r="B108" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="C108" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D108" s="25">
-        <v>55</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A109" s="8" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>191</v>
+        <v>158</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>347</v>
       </c>
       <c r="D109" s="25">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A110" s="8" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>191</v>
+        <v>158</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>273</v>
       </c>
       <c r="D110" s="25">
-        <v>55</v>
+        <v>65</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A111" s="8" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C111" s="5" t="s">
-        <v>191</v>
+        <v>158</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>274</v>
       </c>
       <c r="D111" s="25">
-        <v>55</v>
+        <v>66</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A112" s="8" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B112" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D112" s="25">
-        <v>56</v>
+        <v>67</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A113" s="8" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>194</v>
+        <v>74</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D113" s="25">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A114" s="8" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>86</v>
+        <v>162</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D114" s="25">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A115" s="8" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="D115" s="25">
-        <v>57</v>
+        <v>70</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A116" s="8" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="C116" s="6" t="s">
         <v>277</v>
       </c>
       <c r="D116" s="25">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A117" s="8" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C117" s="5" t="s">
-        <v>287</v>
+        <v>90</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>259</v>
       </c>
       <c r="D117" s="25">
-        <v>59</v>
+        <v>72</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A118" s="8" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>286</v>
+        <v>203</v>
       </c>
       <c r="D118" s="25">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A119" s="8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>202</v>
+        <v>76</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>278</v>
       </c>
       <c r="D119" s="25">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A120" s="8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>210</v>
+        <v>76</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>202</v>
       </c>
       <c r="D120" s="25">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A121" s="8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C121" s="5"/>
-      <c r="D121" s="25"/>
+        <v>88</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D121" s="25">
+        <v>76</v>
+      </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A122" s="8" t="s">
-        <v>157</v>
+        <v>73</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>158</v>
+        <v>74</v>
       </c>
       <c r="C122" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D122" s="25">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A123" s="8" t="s">
-        <v>157</v>
+      <c r="A123" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="C123" s="5" t="s">
         <v>288</v>
       </c>
       <c r="D123" s="25">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A124" s="8" t="s">
-        <v>157</v>
+      <c r="A124" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="C124" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C124" s="5" t="s">
         <v>289</v>
       </c>
       <c r="D124" s="25">
-        <v>64</v>
+        <v>79</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A125" s="8" t="s">
-        <v>157</v>
+      <c r="A125" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="C125" s="6" t="s">
-        <v>279</v>
+        <v>119</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>290</v>
       </c>
       <c r="D125" s="25">
-        <v>66</v>
+        <v>80</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A126" s="8" t="s">
-        <v>157</v>
+      <c r="A126" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="C126" s="5"/>
-      <c r="D126" s="25"/>
+        <v>127</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D126" s="25">
+        <v>81</v>
+      </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A127" s="8" t="s">
-        <v>157</v>
+      <c r="A127" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="C127" s="5"/>
-      <c r="D127" s="25"/>
+        <v>58</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D127" s="25">
+        <v>82</v>
+      </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A128" s="8" t="s">
-        <v>73</v>
+      <c r="A128" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C128" s="6" t="s">
-        <v>280</v>
+        <v>133</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>296</v>
       </c>
       <c r="D128" s="25">
-        <v>68</v>
+        <v>83</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A129" s="8" t="s">
-        <v>73</v>
+      <c r="A129" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="C129" s="6" t="s">
-        <v>263</v>
+        <v>339</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>341</v>
       </c>
       <c r="D129" s="25">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A130" s="8" t="s">
-        <v>73</v>
+      <c r="A130" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="B130" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="D130" s="25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A131" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="D131" s="25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A132" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D132" s="25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A133" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="D133" s="25">
         <v>88</v>
       </c>
-      <c r="C130" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="D130" s="25">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A131" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B131" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C131" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="D131" s="25">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A132" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B132" s="8" t="s">
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A134" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="D134" s="25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A135" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="D135" s="25">
         <v>90</v>
       </c>
-      <c r="C132" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="D132" s="25">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A133" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B133" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C133" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D133" s="25">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A134" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B134" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="C134" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="D134" s="25">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A135" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B135" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C135" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="D135" s="25">
-        <v>74</v>
-      </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A136" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B136" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C136" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="D136" s="25">
-        <v>75</v>
-      </c>
+      <c r="A136" s="5"/>
+      <c r="B136" s="8"/>
+      <c r="C136" s="5"/>
+      <c r="D136" s="25"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A137" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B137" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C137" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="D137" s="25">
-        <v>76</v>
-      </c>
+      <c r="A137" s="5"/>
+      <c r="B137" s="8"/>
+      <c r="C137" s="5"/>
+      <c r="D137" s="25"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A138" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B138" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C138" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="D138" s="25">
-        <v>77</v>
-      </c>
+      <c r="A138" s="5"/>
+      <c r="B138" s="8"/>
+      <c r="C138" s="5"/>
+      <c r="D138" s="25"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A139" s="5"/>
@@ -14483,28 +14489,30 @@
       <c r="C201" s="5"/>
       <c r="D201" s="25"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A202" s="5"/>
-      <c r="B202" s="8"/>
-      <c r="C202" s="5"/>
-      <c r="D202" s="25"/>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A203" s="5"/>
-      <c r="B203" s="8"/>
-      <c r="C203" s="5"/>
-      <c r="D203" s="25"/>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A204" s="5"/>
-      <c r="B204" s="8"/>
-      <c r="C204" s="5"/>
-      <c r="D204" s="25"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D138">
-    <sortCondition ref="A3:A138"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D201">
+    <sortCondition ref="D1:D201"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2F8D84-3B6A-4C1F-B9ED-F757604F663D}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>343</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>